<commit_message>
feat(battle): complete BattleScene content milestone
</commit_message>
<xml_diff>
--- a/DataTables/Datas/battle.card_effect.xlsx
+++ b/DataTables/Datas/battle.card_effect.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Redf4e79157914bb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R3c3d74be5c084791"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -195,7 +195,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="18">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -240,6 +240,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -445,7 +454,7 @@
   <x:cols>
     <x:col min="1" max="1" width="8.75" customWidth="1"/>
     <x:col min="2" max="2" width="9.5" customWidth="1"/>
-    <x:col min="3" max="3" width="15.625" customWidth="1"/>
+    <x:col min="3" max="3" width="24.3799991607666" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="14.25" customWidth="1"/>
     <x:col min="5" max="5" width="6" customWidth="1"/>
   </x:cols>
@@ -591,6 +600,201 @@
         <x:v>3</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11"/>
+      <x:c r="B11" t="n">
+        <x:v>4007</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>DealDamage</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E11" t="n">
+        <x:v>32</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12"/>
+      <x:c r="B12" t="n">
+        <x:v>4008</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>DealDamage</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13"/>
+      <x:c r="B13" t="n">
+        <x:v>4009</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>DealDamage</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E13" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14" t="n">
+        <x:v>4010</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>DrawCards</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E14" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15"/>
+      <x:c r="B15" t="n">
+        <x:v>4011</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>GainBlock</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E15" t="n">
+        <x:v>8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16" t="n">
+        <x:v>4012</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>ExhaustSelectedHandCard</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E16" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17" t="n">
+        <x:v>4013</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>DrawCards</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E17" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18" s="17" t="n">
+        <x:v>4014</x:v>
+      </x:c>
+      <x:c r="C18" s="17" t="str">
+        <x:v>Heal</x:v>
+      </x:c>
+      <x:c r="D18" s="17" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E18" s="17" t="n">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19" t="n">
+        <x:v>4015</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>DealDamage</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E19" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20"/>
+      <x:c r="B20" t="n">
+        <x:v>4016</x:v>
+      </x:c>
+      <x:c r="C20" t="str">
+        <x:v>DealDamageFromSourceBlock</x:v>
+      </x:c>
+      <x:c r="D20" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E20" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21" t="n">
+        <x:v>4017</x:v>
+      </x:c>
+      <x:c r="C21" t="str">
+        <x:v>RetainBlock</x:v>
+      </x:c>
+      <x:c r="D21" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E21" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22"/>
+      <x:c r="B22" t="n">
+        <x:v>4018</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>PlayTopDrawCardAndExhaust</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E22" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23"/>
+      <x:c r="B23" t="n">
+        <x:v>4019</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>RegisterBlockGainRandomEnemyDamage</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="E23" t="n">
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>